<commit_message>
Correo Tania: 18 horas de inasistencia como parte del refuerzo y saldo pendiente de 1.000.000 explicito en ambos caminos
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/experiencia_cliente/Tania/RESPUESTA_TANIA.xlsx
+++ b/recursos/experiencia_cliente/Tania/RESPUESTA_TANIA.xlsx
@@ -480,7 +480,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Una sola condición, y es la más importante: en el refuerzo vas a completar las actividades que quedaron pendientes durante el nivel — los audios, los videos y el proyecto oral. No es un trámite: en tu grupo, los resultados del final siguieron muy de cerca a quienes hicieron esos ejercicios, así fueran de un minuto. Ahí es donde se fija el idioma, y es lo que te va a llevar a pasar el reintento.</t>
+          <t>Una sola condición, y es la más importante: en el refuerzo vas a completar las actividades que quedaron pendientes durante el nivel — los audios, los videos y el proyecto oral — y a cubrir lo visto en las 18 horas de clase a las que no pudiste asistir. No es un trámite: en tu grupo, los resultados del final siguieron muy de cerca a quienes hicieron esos ejercicios, así fueran de un minuto. Ahí es donde se fija el idioma, y es lo que te va a llevar a pasar el reintento.</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Si de todas formas decides retirarte, lo respetamos: te enviamos tu estado de cuenta para dejar todo al día y cerrar con paz y salvo.</t>
+          <t>Sobre tu saldo: en cualquiera de los dos caminos, el valor pendiente de tu programa ($1.000.000) corresponde a lo que ya cursaste y sigue su calendario de pago. Si decides retirarte, lo respetamos: al quedar al día con ese saldo, cerramos con paz y salvo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correo Tania reescrito en la voz de Diana: mas cercano y directo, mismo contenido (recuperacion 300.000, condicion audios/videos/proyecto + 18h, saldo 1.000.000, retiro con paz y salvo)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/experiencia_cliente/Tania/RESPUESTA_TANIA.xlsx
+++ b/recursos/experiencia_cliente/Tania/RESPUESTA_TANIA.xlsx
@@ -429,7 +429,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Buenas tardes, Tania:</t>
+          <t>Hola Tania, ¿cómo estás?</t>
         </is>
       </c>
     </row>
@@ -439,7 +439,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Gracias por escribirnos con tanta claridad y por tu disposición a hacerte responsable. Te respondemos con una buena noticia: no tienes que pagar un nivel completo para recuperar tu A2.</t>
+          <t>Gracias por escribirnos y por ser tan clara. De verdad valoramos mucho que quieras hacerte responsable.</t>
         </is>
       </c>
     </row>
@@ -449,28 +449,28 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Como tu resultado del examen final fue menor a 70/100, calificas para nuestro programa de recuperación del final, que existe justamente para casos como el tuyo:</t>
+          <t>Te tenemos una buena noticia: no tienes que pagar un nivel completo para recuperar tu A2. Como tu examen salió por debajo de 70, puedes entrar a nuestro programa de recuperación del final:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>· 3 sesiones de refuerzo de 2 horas, diseñadas sobre las destrezas donde tu examen salió más bajo.</t>
+          <t>· 3 sesiones de refuerzo de 2 horas, enfocadas justo en lo que más te costó en el examen.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>· 1 reintento del examen final completo, con evaluador externo, en fecha fija.</t>
+          <t>· 1 reintento del examen completo, con evaluador externo.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>· Costo: $300.000, con posibilidad de acuerdo de pago — muy por debajo de lo que costaría repetir el nivel.</t>
+          <t>· Tiene un costo de $300.000, y si lo necesitas te ayudamos con un acuerdo de pago.</t>
         </is>
       </c>
     </row>
@@ -480,7 +480,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Una sola condición, y es la más importante: en el refuerzo vas a completar las actividades que quedaron pendientes durante el nivel — los audios, los videos y el proyecto oral — y a cubrir lo visto en las 18 horas de clase a las que no pudiste asistir. No es un trámite: en tu grupo, los resultados del final siguieron muy de cerca a quienes hicieron esos ejercicios, así fueran de un minuto. Ahí es donde se fija el idioma, y es lo que te va a llevar a pasar el reintento.</t>
+          <t>Eso sí, hay una condición que para nosotros es súper importante: en el refuerzo tienes que hacer los audios, los videos y el proyecto oral que quedaron pendientes, y ponerte al día con lo de las 18 horas de clase a las que no pudiste venir. Y no es por ponerte más trabajo, Tania: la verdad es que en tu grupo, a los que hicieron esos ejercicios —así fueran de un minuto— les fue bien en el final. Es como un nadador: para mejorar hay que meterle horas al agua. Ahí es donde el inglés se queda.</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Es un solo reintento, con la misma exigencia del examen original, para que tu certificado valga lo mismo que el de todos.</t>
+          <t>El reintento es uno solo y con la misma exigencia del examen original, para que tu certificado valga igual que el de todos.</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Sobre tu saldo: en cualquiera de los dos caminos, el valor pendiente de tu programa ($1.000.000) corresponde a lo que ya cursaste y sigue su calendario de pago. Si decides retirarte, lo respetamos: al quedar al día con ese saldo, cerramos con paz y salvo.</t>
+          <t>Sobre tu saldo: el $1.000.000 que tienes pendiente corresponde a lo que ya cursaste, así que sigue su calendario normal en cualquiera de los dos casos. Si al final decides retirarte, lo respetamos, y apenas quedes al día cerramos con paz y salvo.</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Nos encantaría que termines tu A2. ¿Te agendamos la primera sesión de refuerzo? Quedamos atentos.</t>
+          <t>Pero de verdad nos encantaría que termines tu A2 :) ¿Te agendamos la primera sesión de refuerzo?</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Cordialmente,</t>
+          <t>Quedamos atentos, un abrazo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tania final: pago del refuerzo dentro de la proxima cuota (300 refuerzo + 200 programa), sin segunda oportunidad si pierde el reintento, parrafo del medio sin repetir su nombre y mas suave
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/experiencia_cliente/Tania/RESPUESTA_TANIA.xlsx
+++ b/recursos/experiencia_cliente/Tania/RESPUESTA_TANIA.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CORREO TANIA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CORREO TANIA FINAL" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -429,7 +429,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Hola Tania, ¿cómo estás?</t>
+          <t>Hola Tania, esperamos te encuentres bien. Gracias por escribirnos y por ser tan clara. De verdad valoramos mucho cuando nuestros estudiantes toman responsabilidad sobre su proceso. Hemos decidido honrar tu palabra y vamos a darte la oportunidad de tomar el supletorio, así que no tienes que pagar el nivel completo para recuperar tu A2. Sin embargo, ten en cuenta que tu examen salió muy por debajo de 70, y lograr una buena nota con solo tres días de recuperación es un gran reto.</t>
         </is>
       </c>
     </row>
@@ -439,93 +439,90 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Gracias por escribirnos y por ser tan clara. De verdad valoramos mucho que quieras hacerte responsable.</t>
+          <t>El programa de recuperación del examen final consta de:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr"/>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>· 3 sesiones de refuerzo de 2 horas, enfocadas justo en lo que más te costó en el examen.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Te tenemos una buena noticia: no tienes que pagar un nivel completo para recuperar tu A2. Como tu examen salió por debajo de 70, puedes entrar a nuestro programa de recuperación del final:</t>
+          <t>· 1 reintento del examen completo.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>· 3 sesiones de refuerzo de 2 horas, enfocadas justo en lo que más te costó en el examen.</t>
+          <t>· Exposición del proyecto final completo.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>· 1 reintento del examen completo, con evaluador externo.</t>
+          <t>· Tiene un costo de $300.000. Para que no tengas que sacar plata extra, de tu próxima cuota aplicamos $300.000 al refuerzo y $200.000 a tu saldo del programa, y el resto de tu saldo sigue en las cuotas siguientes.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>· Tiene un costo de $300.000, y si lo necesitas te ayudamos con un acuerdo de pago.</t>
-        </is>
-      </c>
+      <c r="A8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Es súper importante que en el refuerzo hagas los audios, los videos y el proyecto oral que quedaron pendientes, y que te pongas al día con lo de las 18 horas de clase a las que no pudiste venir. No es por ponerte más trabajo: son requisitos del programa. En todo el A2 solo enviaste 2 videos, y hacer esos ejercicios, así sean de 1 minuto, es donde tú misma empiezas a coger confianza para hacer las exposiciones. Esto es como cualquier deporte: para ser bueno hay que dedicarle muchas horas en el campo. Sin esos ejercicios, el inglés no avanza.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Eso sí, hay una condición que para nosotros es súper importante: en el refuerzo tienes que hacer los audios, los videos y el proyecto oral que quedaron pendientes, y ponerte al día con lo de las 18 horas de clase a las que no pudiste venir. Y no es por ponerte más trabajo, Tania: la verdad es que en tu grupo, a los que hicieron esos ejercicios —así fueran de un minuto— les fue bien en el final. Es como un nadador: para mejorar hay que meterle horas al agua. Ahí es donde el inglés se queda.</t>
-        </is>
-      </c>
+      <c r="A10" s="1" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr"/>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>El reintento es uno solo y con la misma exigencia del examen original, para que tu certificado valga igual que el de todos. Si en el reintento no alcanzas el 70, no hay otra oportunidad de recuperación.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>El reintento es uno solo y con la misma exigencia del examen original, para que tu certificado valga igual que el de todos.</t>
-        </is>
-      </c>
+      <c r="A12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr"/>
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Sobre tu saldo: el $1.000.000 que tienes pendiente corresponde a lo que ya cursaste, así que sigue su calendario de pago en cualquiera de los dos casos. Si al final decides retirarte, lo respetamos, y apenas quedes al día cerramos con paz y salvo.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Sobre tu saldo: el $1.000.000 que tienes pendiente corresponde a lo que ya cursaste, así que sigue su calendario normal en cualquiera de los dos casos. Si al final decides retirarte, lo respetamos, y apenas quedes al día cerramos con paz y salvo.</t>
-        </is>
-      </c>
+      <c r="A14" s="1" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr"/>
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Pero de verdad nos encantaría que termines tu A2 :) ¿Te agendamos la primera sesión de refuerzo?</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>Pero de verdad nos encantaría que termines tu A2 :) ¿Te agendamos la primera sesión de refuerzo?</t>
-        </is>
-      </c>
+      <c r="A16" s="1" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr"/>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Quedamos atentos, un abrazo.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Quedamos atentos, un abrazo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>Depto. Experiencia al Cliente — Heiiu English Academy</t>
         </is>

</xml_diff>